<commit_message>
Renomeia minicurso de celulas tumorais
</commit_message>
<xml_diff>
--- a/Tabela Minicursos por PPG.xlsx
+++ b/Tabela Minicursos por PPG.xlsx
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Cultivo de células tumorais: da teoria a prática</t>
+          <t>Metabolismo e viabilidade de células tumorais: modelos In vitro e In vivo no estudo do câncer</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Cultivo de células tumorais: da teoria a prática</t>
+          <t>Metabolismo e viabilidade de células tumorais: modelos In vitro e In vivo no estudo do câncer</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ajusta horarios de minicursos
</commit_message>
<xml_diff>
--- a/Tabela Minicursos por PPG.xlsx
+++ b/Tabela Minicursos por PPG.xlsx
@@ -2285,7 +2285,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Terça de manhã Quarta de noite (6h de minicurso)</t>
+          <t>Terça e quarta de noite</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Quarta e Quinta de manhã (8h de minicurso)</t>
+          <t>Quarta e quinta de manhã (4h por dia, 8h totais)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>4 horas</t>
+          <t>8 horas</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza horario dos minicursos noturnos
</commit_message>
<xml_diff>
--- a/Tabela Minicursos por PPG.xlsx
+++ b/Tabela Minicursos por PPG.xlsx
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Terça de noite (3h de minicurso)</t>
+          <t>Terça de noite (18h30-21h30)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Terça e Quarta de noite (6h de minicurso)</t>
+          <t>Terça e quarta de noite (18h30-21h30)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Terça e quarta de noite</t>
+          <t>Terça e quarta de noite (18h30-21h30)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Quarta e Quinta de noite (6h de minicurso)</t>
+          <t>Quarta e quinta de noite (18h30-21h30)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Adiciona popup de aviso: fase de testes - pedidos ate 24/06 15h desconsiderados
</commit_message>
<xml_diff>
--- a/Tabela Minicursos por PPG.xlsx
+++ b/Tabela Minicursos por PPG.xlsx
@@ -1747,7 +1747,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Profa Dra Stephanie Rubianne Silva Carvalhal (PPG-Gen - Fisiologia), Profa MSc Ana Cláudia Thomaz (PPGMICS - UFPR, Nutrição), Profa MSc Ana Paolla Protachevicz (PPGCF - UEPG), MSc. Fernanda Vitório da Silva (PPG-Gen), Raphaela Ohana Rios.</t>
+          <t>Profa Dra Stephanie Rubianne Silva Carvalhal (PPG-Gen - Fisiologia), Profa MSc Ana Cláudia Thomaz (PPGMICS - UFPR, Nutrição), Profa MSc Ana Paolla Protachevicz (PPGCF - UEPG), MSc. Fernanda Vitório da Silva (PPG-Gen), Profa. Especialista Raphaela Ohanna Schmitz Rios.</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Profa Dra Stephanie Rubianne Silva Carvalhal (PPG-Gen - Fisiologia), Profa MSc Ana Cláudia Thomaz (PPGMICS - UFPR, Nutrição), Profa MSc Ana Paolla Protachevicz (PPGCF - UEPG), MSc. Fernanda Vitório da Silva (PPG-Gen), Raphaela Ohana Rios.</t>
+          <t>Profa Dra Stephanie Rubianne Silva Carvalhal (PPG-Gen - Fisiologia), Profa MSc Ana Cláudia Thomaz (PPGMICS - UFPR, Nutrição), Profa MSc Ana Paolla Protachevicz (PPGCF - UEPG), MSc. Fernanda Vitório da Silva (PPG-Gen), Profa. Especialista Raphaela Ohanna Schmitz Rios.</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualiza vagas ilimitadas do DOHAD
</commit_message>
<xml_diff>
--- a/Tabela Minicursos por PPG.xlsx
+++ b/Tabela Minicursos por PPG.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Todos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Genetica" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Biocel" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Bioquimica" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Genetica" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biocel" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bioquimica" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todos'!$A$1:$T$24</definedName>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>Ilimitadas</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza vagas e endpoint do Apps Script
</commit_message>
<xml_diff>
--- a/Tabela Minicursos por PPG.xlsx
+++ b/Tabela Minicursos por PPG.xlsx
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>